<commit_message>
refactor(docs): 按钮 sheet 精简，去掉 条件JSON/消耗JSON/效果JSON 三列
- gen-config-template.mjs: H_BTN 10→7列(关联节点中文名/序号/文案/类型/必现/权重/目标中文名)，mkBtn 删三行 set
- export-db-to-excel.mjs: H_BTN 与 btn_rows 构造同步精简
- resolve-config.mjs 按钮逻辑按列名动态索引，自动适配无需改
- admin-api.md §18 按钮行、MEMORY.md Excel 段同步去掉三 JSON 列
- 管道验证：模板/导出按钮 7 列、已解析版 8 列(+目标code)，0 错误
</commit_message>
<xml_diff>
--- a/剧情配置/事件与节点配置表.xlsx
+++ b/剧情配置/事件与节点配置表.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="58">
   <si>
     <t>中文名</t>
   </si>
@@ -163,15 +163,6 @@
   </si>
   <si>
     <t>权重</t>
-  </si>
-  <si>
-    <t>条件JSON</t>
-  </si>
-  <si>
-    <t>消耗JSON</t>
-  </si>
-  <si>
-    <t>效果JSON</t>
   </si>
   <si>
     <t>目标中文名</t>
@@ -890,13 +881,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="10" width="13" customWidth="1"/>
+    <col min="1" max="7" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>44</v>
       </c>
@@ -918,28 +909,19 @@
       <c r="G1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C2" t="s">
         <v>27</v>
       </c>
       <c r="D2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E2" t="s">
         <v>25</v>
@@ -948,30 +930,21 @@
         <v>6</v>
       </c>
       <c r="G2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" t="s">
-        <v>6</v>
-      </c>
-      <c r="I2" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
         <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E3" t="s">
         <v>25</v>
@@ -980,19 +953,10 @@
         <v>6</v>
       </c>
       <c r="G3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" t="s">
-        <v>6</v>
-      </c>
-      <c r="I3" t="s">
-        <v>6</v>
-      </c>
-      <c r="J3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1000,10 +964,10 @@
         <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E4" t="s">
         <v>25</v>
@@ -1012,30 +976,21 @@
         <v>6</v>
       </c>
       <c r="G4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H4" t="s">
-        <v>6</v>
-      </c>
-      <c r="I4" t="s">
-        <v>6</v>
-      </c>
-      <c r="J4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E5" t="s">
         <v>25</v>
@@ -1044,30 +999,21 @@
         <v>6</v>
       </c>
       <c r="G5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H5" t="s">
-        <v>6</v>
-      </c>
-      <c r="I5" t="s">
-        <v>6</v>
-      </c>
-      <c r="J5" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D6" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E6" t="s">
         <v>25</v>
@@ -1076,30 +1022,21 @@
         <v>6</v>
       </c>
       <c r="G6" t="s">
-        <v>6</v>
-      </c>
-      <c r="H6" t="s">
-        <v>6</v>
-      </c>
-      <c r="I6" t="s">
-        <v>6</v>
-      </c>
-      <c r="J6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D7" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E7" t="s">
         <v>25</v>
@@ -1108,30 +1045,21 @@
         <v>6</v>
       </c>
       <c r="G7" t="s">
-        <v>6</v>
-      </c>
-      <c r="H7" t="s">
-        <v>6</v>
-      </c>
-      <c r="I7" t="s">
-        <v>6</v>
-      </c>
-      <c r="J7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>41</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C8" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D8" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E8" t="s">
         <v>25</v>
@@ -1140,15 +1068,6 @@
         <v>6</v>
       </c>
       <c r="G8" t="s">
-        <v>6</v>
-      </c>
-      <c r="H8" t="s">
-        <v>6</v>
-      </c>
-      <c r="I8" t="s">
-        <v>6</v>
-      </c>
-      <c r="J8" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>